<commit_message>
Update benchmark CGRI scores in Excel with new 20/40/40 weights
</commit_message>
<xml_diff>
--- a/data/processed/Template CGRI.xlsx
+++ b/data/processed/Template CGRI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arzumkarahan/Desktop/DSBA/2nd year/Geopolitics/Group Project/company-geopolitical-risk-index/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439467C4-65B8-9D4A-B536-2F2C4B48D0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB1CEC0-A852-1842-8950-07C275203FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="18000" xr2:uid="{266D4EF2-EDBA-FA44-A696-554C257F20B6}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{266D4EF2-EDBA-FA44-A696-554C257F20B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -1553,8 +1553,53 @@
     <xf numFmtId="0" fontId="15" fillId="16" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1589,53 +1634,8 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -3990,37 +3990,35 @@
       <sheetName val="Country of Revenues - Toyota"/>
       <sheetName val="Country of Revenues - TSMC"/>
       <sheetName val="Country of Revenues - VW"/>
-      <sheetName val="Revenue Exposure"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -4060,37 +4058,35 @@
       <sheetName val="Country of Suppliers - Samsung"/>
       <sheetName val="Country of Suppliers - Amazon"/>
       <sheetName val="Country of Suppliers - Ford"/>
-      <sheetName val="Supply Chain Exposure"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -4629,42 +4625,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="113" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="100"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
+      <c r="H1" s="114"/>
+      <c r="I1" s="114"/>
+      <c r="J1" s="114"/>
+      <c r="K1" s="114"/>
+      <c r="L1" s="114"/>
+      <c r="M1" s="114"/>
+      <c r="N1" s="114"/>
+      <c r="O1" s="114"/>
+      <c r="P1" s="114"/>
+      <c r="Q1" s="114"/>
+      <c r="R1" s="115"/>
     </row>
     <row r="2" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="96"/>
-      <c r="B2" s="97"/>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="97"/>
-      <c r="L2" s="97"/>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
+      <c r="A2" s="111"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="112"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="112"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
       <c r="O2" s="28"/>
       <c r="P2" s="28"/>
       <c r="Q2" s="28"/>
@@ -4799,19 +4795,19 @@
       <c r="R8" s="36"/>
     </row>
     <row r="9" spans="1:19" ht="25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="105" t="s">
+      <c r="A9" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="106"/>
-      <c r="C9" s="106"/>
-      <c r="D9" s="106"/>
-      <c r="E9" s="106"/>
-      <c r="F9" s="106"/>
-      <c r="G9" s="106"/>
-      <c r="H9" s="106"/>
-      <c r="I9" s="106"/>
-      <c r="J9" s="106"/>
-      <c r="K9" s="106"/>
+      <c r="B9" s="121"/>
+      <c r="C9" s="121"/>
+      <c r="D9" s="121"/>
+      <c r="E9" s="121"/>
+      <c r="F9" s="121"/>
+      <c r="G9" s="121"/>
+      <c r="H9" s="121"/>
+      <c r="I9" s="121"/>
+      <c r="J9" s="121"/>
+      <c r="K9" s="121"/>
       <c r="L9" s="37"/>
       <c r="M9" s="37"/>
       <c r="N9" s="37"/>
@@ -4821,12 +4817,12 @@
       <c r="R9" s="38"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A10" s="101" t="s">
+      <c r="A10" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="102"/>
-      <c r="C10" s="102"/>
-      <c r="D10" s="102"/>
+      <c r="B10" s="117"/>
+      <c r="C10" s="117"/>
+      <c r="D10" s="117"/>
       <c r="E10" s="37"/>
       <c r="F10" s="37"/>
       <c r="G10" s="37"/>
@@ -4843,10 +4839,10 @@
       <c r="R10" s="38"/>
     </row>
     <row r="11" spans="1:19" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="103"/>
-      <c r="B11" s="104"/>
-      <c r="C11" s="104"/>
-      <c r="D11" s="104"/>
+      <c r="A11" s="118"/>
+      <c r="B11" s="119"/>
+      <c r="C11" s="119"/>
+      <c r="D11" s="119"/>
       <c r="E11" s="39"/>
       <c r="F11" s="39"/>
       <c r="G11" s="39"/>
@@ -4883,17 +4879,17 @@
       <c r="R12" s="49"/>
     </row>
     <row r="13" spans="1:19" ht="22" x14ac:dyDescent="0.3">
-      <c r="A13" s="107" t="s">
+      <c r="A13" s="103" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="108"/>
-      <c r="C13" s="108"/>
-      <c r="D13" s="108"/>
-      <c r="E13" s="108"/>
-      <c r="F13" s="108"/>
-      <c r="G13" s="108"/>
-      <c r="H13" s="108"/>
-      <c r="I13" s="108"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="104"/>
+      <c r="F13" s="104"/>
+      <c r="G13" s="104"/>
+      <c r="H13" s="104"/>
+      <c r="I13" s="104"/>
       <c r="J13" s="50"/>
       <c r="K13" s="50"/>
       <c r="L13" s="50"/>
@@ -4945,24 +4941,24 @@
       <c r="R15" s="49"/>
     </row>
     <row r="16" spans="1:19" ht="22" x14ac:dyDescent="0.3">
-      <c r="A16" s="107" t="s">
+      <c r="A16" s="103" t="s">
         <v>146</v>
       </c>
-      <c r="B16" s="108"/>
-      <c r="C16" s="108"/>
-      <c r="D16" s="108"/>
-      <c r="E16" s="108"/>
-      <c r="F16" s="108"/>
-      <c r="G16" s="108"/>
-      <c r="H16" s="108"/>
-      <c r="I16" s="108"/>
-      <c r="J16" s="108"/>
-      <c r="K16" s="108"/>
-      <c r="L16" s="108"/>
-      <c r="M16" s="108"/>
-      <c r="N16" s="108"/>
-      <c r="O16" s="108"/>
-      <c r="P16" s="108"/>
+      <c r="B16" s="104"/>
+      <c r="C16" s="104"/>
+      <c r="D16" s="104"/>
+      <c r="E16" s="104"/>
+      <c r="F16" s="104"/>
+      <c r="G16" s="104"/>
+      <c r="H16" s="104"/>
+      <c r="I16" s="104"/>
+      <c r="J16" s="104"/>
+      <c r="K16" s="104"/>
+      <c r="L16" s="104"/>
+      <c r="M16" s="104"/>
+      <c r="N16" s="104"/>
+      <c r="O16" s="104"/>
+      <c r="P16" s="104"/>
       <c r="Q16" s="48"/>
       <c r="R16" s="49"/>
     </row>
@@ -5007,26 +5003,26 @@
       <c r="R18" s="49"/>
     </row>
     <row r="19" spans="1:32" ht="22" x14ac:dyDescent="0.3">
-      <c r="A19" s="107" t="s">
+      <c r="A19" s="103" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="108"/>
-      <c r="C19" s="108"/>
-      <c r="D19" s="108"/>
-      <c r="E19" s="108"/>
-      <c r="F19" s="108"/>
-      <c r="G19" s="108"/>
-      <c r="H19" s="108"/>
-      <c r="I19" s="108"/>
-      <c r="J19" s="108"/>
-      <c r="K19" s="108"/>
-      <c r="L19" s="108"/>
-      <c r="M19" s="108"/>
-      <c r="N19" s="108"/>
-      <c r="O19" s="108"/>
-      <c r="P19" s="108"/>
-      <c r="Q19" s="108"/>
-      <c r="R19" s="117"/>
+      <c r="B19" s="104"/>
+      <c r="C19" s="104"/>
+      <c r="D19" s="104"/>
+      <c r="E19" s="104"/>
+      <c r="F19" s="104"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="104"/>
+      <c r="I19" s="104"/>
+      <c r="J19" s="104"/>
+      <c r="K19" s="104"/>
+      <c r="L19" s="104"/>
+      <c r="M19" s="104"/>
+      <c r="N19" s="104"/>
+      <c r="O19" s="104"/>
+      <c r="P19" s="104"/>
+      <c r="Q19" s="104"/>
+      <c r="R19" s="105"/>
     </row>
     <row r="20" spans="1:32" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="51"/>
@@ -5111,23 +5107,23 @@
       <c r="R23" s="41"/>
     </row>
     <row r="24" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="118"/>
-      <c r="B24" s="119"/>
-      <c r="C24" s="119"/>
-      <c r="D24" s="119"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
-      <c r="G24" s="119"/>
-      <c r="H24" s="119"/>
-      <c r="I24" s="119"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="119"/>
-      <c r="L24" s="119"/>
-      <c r="M24" s="119"/>
-      <c r="N24" s="119"/>
-      <c r="O24" s="119"/>
-      <c r="P24" s="119"/>
-      <c r="Q24" s="119"/>
+      <c r="A24" s="106"/>
+      <c r="B24" s="107"/>
+      <c r="C24" s="107"/>
+      <c r="D24" s="107"/>
+      <c r="E24" s="107"/>
+      <c r="F24" s="107"/>
+      <c r="G24" s="107"/>
+      <c r="H24" s="107"/>
+      <c r="I24" s="107"/>
+      <c r="J24" s="107"/>
+      <c r="K24" s="107"/>
+      <c r="L24" s="107"/>
+      <c r="M24" s="107"/>
+      <c r="N24" s="107"/>
+      <c r="O24" s="107"/>
+      <c r="P24" s="107"/>
+      <c r="Q24" s="107"/>
       <c r="R24" s="54"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
@@ -5145,164 +5141,164 @@
       <c r="AF24" s="4"/>
     </row>
     <row r="25" spans="1:32" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="120" t="s">
+      <c r="A25" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="121"/>
-      <c r="C25" s="121"/>
-      <c r="D25" s="121"/>
-      <c r="E25" s="121"/>
-      <c r="F25" s="121"/>
-      <c r="G25" s="121"/>
-      <c r="H25" s="121"/>
-      <c r="I25" s="121"/>
-      <c r="J25" s="121"/>
-      <c r="K25" s="121"/>
-      <c r="L25" s="121"/>
-      <c r="M25" s="121"/>
-      <c r="N25" s="121"/>
-      <c r="O25" s="121"/>
-      <c r="P25" s="121"/>
-      <c r="Q25" s="121"/>
-      <c r="R25" s="122"/>
+      <c r="B25" s="109"/>
+      <c r="C25" s="109"/>
+      <c r="D25" s="109"/>
+      <c r="E25" s="109"/>
+      <c r="F25" s="109"/>
+      <c r="G25" s="109"/>
+      <c r="H25" s="109"/>
+      <c r="I25" s="109"/>
+      <c r="J25" s="109"/>
+      <c r="K25" s="109"/>
+      <c r="L25" s="109"/>
+      <c r="M25" s="109"/>
+      <c r="N25" s="109"/>
+      <c r="O25" s="109"/>
+      <c r="P25" s="109"/>
+      <c r="Q25" s="109"/>
+      <c r="R25" s="110"/>
     </row>
     <row r="26" spans="1:32" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="120"/>
-      <c r="B26" s="121"/>
-      <c r="C26" s="121"/>
-      <c r="D26" s="121"/>
-      <c r="E26" s="121"/>
-      <c r="F26" s="121"/>
-      <c r="G26" s="121"/>
-      <c r="H26" s="121"/>
-      <c r="I26" s="121"/>
-      <c r="J26" s="121"/>
-      <c r="K26" s="121"/>
-      <c r="L26" s="121"/>
-      <c r="M26" s="121"/>
-      <c r="N26" s="121"/>
-      <c r="O26" s="121"/>
-      <c r="P26" s="121"/>
-      <c r="Q26" s="121"/>
-      <c r="R26" s="122"/>
+      <c r="A26" s="108"/>
+      <c r="B26" s="109"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="109"/>
+      <c r="G26" s="109"/>
+      <c r="H26" s="109"/>
+      <c r="I26" s="109"/>
+      <c r="J26" s="109"/>
+      <c r="K26" s="109"/>
+      <c r="L26" s="109"/>
+      <c r="M26" s="109"/>
+      <c r="N26" s="109"/>
+      <c r="O26" s="109"/>
+      <c r="P26" s="109"/>
+      <c r="Q26" s="109"/>
+      <c r="R26" s="110"/>
     </row>
     <row r="27" spans="1:32" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="109" t="s">
+      <c r="A27" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="110"/>
-      <c r="C27" s="110"/>
-      <c r="D27" s="110"/>
-      <c r="E27" s="110"/>
-      <c r="F27" s="110"/>
-      <c r="G27" s="110"/>
-      <c r="H27" s="110"/>
-      <c r="I27" s="110"/>
-      <c r="J27" s="110"/>
-      <c r="K27" s="110"/>
-      <c r="L27" s="110"/>
-      <c r="M27" s="110"/>
-      <c r="N27" s="110"/>
-      <c r="O27" s="110"/>
-      <c r="P27" s="110"/>
-      <c r="Q27" s="110"/>
-      <c r="R27" s="111"/>
+      <c r="B27" s="96"/>
+      <c r="C27" s="96"/>
+      <c r="D27" s="96"/>
+      <c r="E27" s="96"/>
+      <c r="F27" s="96"/>
+      <c r="G27" s="96"/>
+      <c r="H27" s="96"/>
+      <c r="I27" s="96"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="96"/>
+      <c r="L27" s="96"/>
+      <c r="M27" s="96"/>
+      <c r="N27" s="96"/>
+      <c r="O27" s="96"/>
+      <c r="P27" s="96"/>
+      <c r="Q27" s="96"/>
+      <c r="R27" s="97"/>
     </row>
     <row r="28" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="109"/>
-      <c r="B28" s="110"/>
-      <c r="C28" s="110"/>
-      <c r="D28" s="110"/>
-      <c r="E28" s="110"/>
-      <c r="F28" s="110"/>
-      <c r="G28" s="110"/>
-      <c r="H28" s="110"/>
-      <c r="I28" s="110"/>
-      <c r="J28" s="110"/>
-      <c r="K28" s="110"/>
-      <c r="L28" s="110"/>
-      <c r="M28" s="110"/>
-      <c r="N28" s="110"/>
-      <c r="O28" s="110"/>
-      <c r="P28" s="110"/>
-      <c r="Q28" s="110"/>
-      <c r="R28" s="111"/>
+      <c r="A28" s="95"/>
+      <c r="B28" s="96"/>
+      <c r="C28" s="96"/>
+      <c r="D28" s="96"/>
+      <c r="E28" s="96"/>
+      <c r="F28" s="96"/>
+      <c r="G28" s="96"/>
+      <c r="H28" s="96"/>
+      <c r="I28" s="96"/>
+      <c r="J28" s="96"/>
+      <c r="K28" s="96"/>
+      <c r="L28" s="96"/>
+      <c r="M28" s="96"/>
+      <c r="N28" s="96"/>
+      <c r="O28" s="96"/>
+      <c r="P28" s="96"/>
+      <c r="Q28" s="96"/>
+      <c r="R28" s="97"/>
     </row>
     <row r="29" spans="1:32" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="109"/>
-      <c r="B29" s="110"/>
-      <c r="C29" s="110"/>
-      <c r="D29" s="110"/>
-      <c r="E29" s="110"/>
-      <c r="F29" s="110"/>
-      <c r="G29" s="110"/>
-      <c r="H29" s="110"/>
-      <c r="I29" s="110"/>
-      <c r="J29" s="110"/>
-      <c r="K29" s="110"/>
-      <c r="L29" s="110"/>
-      <c r="M29" s="110"/>
-      <c r="N29" s="110"/>
-      <c r="O29" s="110"/>
-      <c r="P29" s="110"/>
-      <c r="Q29" s="110"/>
-      <c r="R29" s="111"/>
+      <c r="A29" s="95"/>
+      <c r="B29" s="96"/>
+      <c r="C29" s="96"/>
+      <c r="D29" s="96"/>
+      <c r="E29" s="96"/>
+      <c r="F29" s="96"/>
+      <c r="G29" s="96"/>
+      <c r="H29" s="96"/>
+      <c r="I29" s="96"/>
+      <c r="J29" s="96"/>
+      <c r="K29" s="96"/>
+      <c r="L29" s="96"/>
+      <c r="M29" s="96"/>
+      <c r="N29" s="96"/>
+      <c r="O29" s="96"/>
+      <c r="P29" s="96"/>
+      <c r="Q29" s="96"/>
+      <c r="R29" s="97"/>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A30" s="112" t="s">
+      <c r="A30" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="B30" s="113"/>
-      <c r="C30" s="113"/>
-      <c r="D30" s="113"/>
-      <c r="E30" s="113"/>
-      <c r="F30" s="113"/>
-      <c r="G30" s="113"/>
-      <c r="H30" s="113"/>
-      <c r="I30" s="113"/>
-      <c r="J30" s="113"/>
-      <c r="K30" s="113"/>
-      <c r="L30" s="113"/>
-      <c r="M30" s="113"/>
-      <c r="N30" s="113"/>
-      <c r="O30" s="113"/>
-      <c r="P30" s="113"/>
-      <c r="Q30" s="113"/>
-      <c r="R30" s="114"/>
+      <c r="B30" s="99"/>
+      <c r="C30" s="99"/>
+      <c r="D30" s="99"/>
+      <c r="E30" s="99"/>
+      <c r="F30" s="99"/>
+      <c r="G30" s="99"/>
+      <c r="H30" s="99"/>
+      <c r="I30" s="99"/>
+      <c r="J30" s="99"/>
+      <c r="K30" s="99"/>
+      <c r="L30" s="99"/>
+      <c r="M30" s="99"/>
+      <c r="N30" s="99"/>
+      <c r="O30" s="99"/>
+      <c r="P30" s="99"/>
+      <c r="Q30" s="99"/>
+      <c r="R30" s="100"/>
     </row>
     <row r="31" spans="1:32" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="115"/>
-      <c r="B31" s="115"/>
-      <c r="C31" s="115"/>
-      <c r="D31" s="115"/>
-      <c r="E31" s="115"/>
-      <c r="F31" s="115"/>
-      <c r="G31" s="115"/>
-      <c r="H31" s="115"/>
-      <c r="I31" s="115"/>
-      <c r="J31" s="115"/>
-      <c r="K31" s="115"/>
-      <c r="L31" s="115"/>
-      <c r="M31" s="115"/>
-      <c r="N31" s="115"/>
-      <c r="O31" s="115"/>
-      <c r="P31" s="115"/>
-      <c r="Q31" s="115"/>
-      <c r="R31" s="116"/>
+      <c r="A31" s="101"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="101"/>
+      <c r="E31" s="101"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="101"/>
+      <c r="H31" s="101"/>
+      <c r="I31" s="101"/>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="101"/>
+      <c r="Q31" s="101"/>
+      <c r="R31" s="102"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A10:D11"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="A13:I13"/>
     <mergeCell ref="A27:R29"/>
     <mergeCell ref="A30:R31"/>
     <mergeCell ref="A16:P16"/>
     <mergeCell ref="A19:R19"/>
     <mergeCell ref="A24:Q24"/>
     <mergeCell ref="A25:R26"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A10:D11"/>
-    <mergeCell ref="A9:K9"/>
-    <mergeCell ref="A13:I13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5329,17 +5325,17 @@
   <sheetData>
     <row r="1" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11"/>
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="122" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
       <c r="E1" s="94"/>
-      <c r="F1" s="95" t="s">
+      <c r="F1" s="122" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
       <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -5397,8 +5393,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H3" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.2329977178729381</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.2341629210672878</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -5430,8 +5426,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H4" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>4.20040509952522</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>4.1224201273946832</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -5463,8 +5459,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H5" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.3492023453852702</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.3527009387433941</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -5496,8 +5492,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H6" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.3708271672512238</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.3370317187938516</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -5529,8 +5525,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H7" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.9423810394738572</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.9590017074492954</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -5562,8 +5558,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H8" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.3623470485532048</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.3659147915694292</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -5595,8 +5591,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H9" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.5146561371664067</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.5101763308337643</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,8 +5624,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H10" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.6108798837735678</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.5735273258773814</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -5661,8 +5657,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H11" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.7381580746102783</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.7031493026055951</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -5694,8 +5690,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H12" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>2.714839155854162</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>2.7014553727535269</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -5727,8 +5723,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H13" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.1862337233911346</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.1689434997969013</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -5760,8 +5756,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H14" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>2.922946008700579</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>2.927222753446685</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -5793,8 +5789,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H15" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.8689896052884483</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.8259774068860732</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -5826,8 +5822,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H16" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.0111654637861411</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>2.9406831938015419</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -5859,8 +5855,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H17" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.8043721298581952</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.7603096388070711</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -5892,8 +5888,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H18" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.1054044035090187</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.0913553768712871</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -5925,8 +5921,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H19" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>5.646494063119821</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>5.5404198631744634</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -5958,8 +5954,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H20" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.2333252749144665</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.2143833396415848</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -5991,8 +5987,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H21" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.1143484151847991</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.1077680719530325</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -6024,8 +6020,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H22" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.242332808890394</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.2191176467995981</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -6057,8 +6053,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H23" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>4.7016474234051842</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>4.6123039334998115</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -6090,8 +6086,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H24" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.2967671490720662</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.3049083714544709</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -6123,8 +6119,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H25" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>3.0895514355683051</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>3.0635163871469113</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -6156,8 +6152,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H26" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>4.1359178283459732</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>4.0539948771988161</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -6189,8 +6185,8 @@
         <v>0.9348282637706109</v>
       </c>
       <c r="H27" s="13">
-        <f>(0.15*Tabella6[[#This Row],[HQ Country Risk]]+0.45*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
-        <v>2.9045955305767293</v>
+        <f>(0.2*Tabella6[[#This Row],[HQ Country Risk]]+0.4*Tabella6[[#This Row],[Revenue Exposure]]+0.4*Tabella6[[#This Row],[Supply Chain Exposure]])*Tabella6[[#This Row],[Financial Exposure]]*Tabella6[[#This Row],[Sector Risk]]*Tabella6[[#This Row],[Volatility Risk]]</f>
+        <v>2.9042897821266824</v>
       </c>
     </row>
   </sheetData>
@@ -61758,18 +61754,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -61791,18 +61787,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E6D44B9-BFA0-496F-91FF-88181837C605}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D57F7E9-094C-4E40-AC1D-B397B1E486C4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E6D44B9-BFA0-496F-91FF-88181837C605}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>